<commit_message>
The royalty case's members add up to what they share, cent for cent, and it names what rests on the duplicate and what the deduction does not say: split by the largest remainder the label's debt is 2,410.15 across four people, not 2,410.17; 68.48 of it rests on Deezer's double report, which moved the recoupment; and the EP deduction, which takes more streams than its month counted, is a question for the distributor rather than streams called artificial
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/label-royalties/royalties.xlsx
+++ b/samples/label-royalties/royalties.xlsx
@@ -1487,11 +1487,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jonas Brandt</t>
+          <t>Mara Keller</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3180.98</v>
+        <v>3277.37</v>
       </c>
       <c r="C2" t="n">
         <v>199.89</v>
@@ -1500,64 +1500,64 @@
         <v>723.05</v>
       </c>
       <c r="E2" t="n">
-        <v>4103.92</v>
+        <v>4200.31</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lena Ortiz (producer)</t>
+          <t>Jonas Brandt</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>3180.98</v>
       </c>
       <c r="C3" t="n">
-        <v>66.63</v>
+        <v>199.89</v>
       </c>
       <c r="D3" t="n">
-        <v>241.02</v>
+        <v>723.05</v>
       </c>
       <c r="E3" t="n">
-        <v>307.65</v>
+        <v>4103.92</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mara Keller</t>
+          <t>Teo Vasić</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3277.37</v>
+        <v>3180.97</v>
       </c>
       <c r="C4" t="n">
-        <v>199.89</v>
+        <v>199.88</v>
       </c>
       <c r="D4" t="n">
-        <v>723.05</v>
+        <v>723.04</v>
       </c>
       <c r="E4" t="n">
-        <v>4200.31</v>
+        <v>4103.89</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Teo Vasić</t>
+          <t>Lena Ortiz (producer)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3180.98</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>199.89</v>
+        <v>66.63</v>
       </c>
       <c r="D5" t="n">
-        <v>723.05</v>
+        <v>241.01</v>
       </c>
       <c r="E5" t="n">
-        <v>4103.92</v>
+        <v>307.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>